<commit_message>
🔄 MAJ automatique BRVM via GitHub Actions
</commit_message>
<xml_diff>
--- a/data/recommandations.xlsx
+++ b/data/recommandations.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,10 +476,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>2033.06</v>
+        <v>1624.92</v>
       </c>
       <c r="E2" t="n">
         <v>407.43</v>
@@ -505,10 +505,10 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>1506.42</v>
+        <v>1207.79</v>
       </c>
       <c r="E3" t="n">
         <v>297.67</v>
@@ -534,10 +534,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>1402.32</v>
+        <v>1118.68</v>
       </c>
       <c r="E4" t="n">
         <v>281.52</v>
@@ -563,10 +563,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>1298.3</v>
+        <v>1037.24</v>
       </c>
       <c r="E5" t="n">
         <v>259.68</v>
@@ -592,10 +592,10 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>1164.88</v>
+        <v>929.6</v>
       </c>
       <c r="E6" t="n">
         <v>232.1</v>
@@ -621,10 +621,10 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>1112.19</v>
+        <v>889.6</v>
       </c>
       <c r="E7" t="n">
         <v>223.6</v>
@@ -650,10 +650,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>1064.11</v>
+        <v>849.98</v>
       </c>
       <c r="E8" t="n">
         <v>212.59</v>
@@ -679,10 +679,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>1003.81</v>
+        <v>802.84</v>
       </c>
       <c r="E9" t="n">
         <v>201.81</v>
@@ -708,10 +708,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>884.84</v>
+        <v>710.53</v>
       </c>
       <c r="E10" t="n">
         <v>179.38</v>
@@ -737,10 +737,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>713.04</v>
+        <v>571.5</v>
       </c>
       <c r="E11" t="n">
         <v>144.53</v>
@@ -759,7 +759,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BANK OF AFRICA ML (BOAM)</t>
+          <t>SMB CI (SMBC)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -769,10 +769,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>10.05</v>
+        <v>4.88</v>
       </c>
       <c r="E12" t="n">
-        <v>2.71</v>
+        <v>2.81</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NSIA BANQUE COTE D'IVOIRE (NSBC)</t>
+          <t>ERIUM CI (Ex AIR LIQUIDE CI) (SIVC)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -798,10 +798,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>7.49</v>
+        <v>4.35</v>
       </c>
       <c r="E13" t="n">
-        <v>7.49</v>
+        <v>4.35</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -817,20 +817,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORANGE COTE D'IVOIRE (ORAC)</t>
+          <t>UNILEVER CI (UNLC)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>6.77</v>
+        <v>3.72</v>
       </c>
       <c r="E14" t="n">
-        <v>3.01</v>
+        <v>3.72</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -846,20 +846,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SMB CI (SMBC)</t>
+          <t>BERNABE CI (BNBC)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>4.88</v>
+        <v>3.67</v>
       </c>
       <c r="E15" t="n">
-        <v>2.81</v>
+        <v>3.67</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -875,20 +875,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CIE CI (CIEC)</t>
+          <t>TRACTAFRIC MOTORS CI (PRSC)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>4.66</v>
+        <v>3.33</v>
       </c>
       <c r="E16" t="n">
-        <v>-4.05</v>
+        <v>3.33</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -897,14 +897,14 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ERIUM CI (Ex AIR LIQUIDE CI) (SIVC)</t>
+          <t>SETAO CI (STAC)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -914,10 +914,10 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>4.35</v>
+        <v>3.2</v>
       </c>
       <c r="E17" t="n">
-        <v>4.35</v>
+        <v>3.2</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BERNABE CI (BNBC)</t>
+          <t>ORANGE COTE D'IVOIRE (ORAC)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -943,10 +943,10 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>3.67</v>
+        <v>3.01</v>
       </c>
       <c r="E18" t="n">
-        <v>3.67</v>
+        <v>3.01</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TRACTAFRIC MOTORS CI (PRSC)</t>
+          <t>BANK OF AFRICA ML (BOAM)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -972,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>3.33</v>
+        <v>2.71</v>
       </c>
       <c r="E19" t="n">
-        <v>3.33</v>
+        <v>2.71</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -991,20 +991,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SETAO CI (STAC)</t>
+          <t>LOTERIE NATIONALE DU BENIN (LNBB)</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>3.2</v>
+        <v>2.66</v>
       </c>
       <c r="E20" t="n">
-        <v>3.2</v>
+        <v>-2.47</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>➖ Neutre</t>
+          <t>👀 À surveiller</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NESTLE CI (NTLC)</t>
+          <t>EVIOSYS PACKAGING SIEM CI (SEMC)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1117,10 +1117,10 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>0.4</v>
+        <v>0.18</v>
       </c>
       <c r="E24" t="n">
-        <v>-6.11</v>
+        <v>4.33</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1136,7 +1136,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EVIOSYS PACKAGING SIEM CI (SEMC)</t>
+          <t>BIIC BN (BICB)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1146,10 +1146,10 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0.18</v>
+        <v>-0.8</v>
       </c>
       <c r="E25" t="n">
-        <v>4.33</v>
+        <v>2.45</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1165,7 +1165,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BIIC BN (BICB)</t>
+          <t>CIE CI (CIEC)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1175,10 +1175,10 @@
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.8</v>
+        <v>-1.01</v>
       </c>
       <c r="E26" t="n">
-        <v>2.45</v>
+        <v>-4.05</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1194,20 +1194,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LOTERIE NATIONALE DU BENIN (LNBB)</t>
+          <t>AFRICA GLOBAL LOGISTICS CI (SDSC)</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>-1.04</v>
+        <v>-1.94</v>
       </c>
       <c r="E27" t="n">
-        <v>-2.47</v>
+        <v>-1.94</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1216,14 +1216,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AFRICA GLOBAL LOGISTICS CI (SDSC)</t>
+          <t>SODE CI (SDCC)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1233,10 +1233,10 @@
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>-1.94</v>
+        <v>-2</v>
       </c>
       <c r="E28" t="n">
-        <v>-1.94</v>
+        <v>-2</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1252,20 +1252,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SODE CI (SDCC)</t>
+          <t>ECOBANK COTE D''IVOIRE (ECOC)</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>-2</v>
+        <v>-2.17</v>
       </c>
       <c r="E29" t="n">
-        <v>-2</v>
+        <v>2.89</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1274,27 +1274,27 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>➖ Neutre</t>
+          <t>👀 À surveiller</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ECOBANK COTE D''IVOIRE (ECOC)</t>
+          <t>NEI-CEDA CI (NEIC)</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>-2.17</v>
+        <v>-2.63</v>
       </c>
       <c r="E30" t="n">
-        <v>2.89</v>
+        <v>-2.65</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1310,20 +1310,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>UNILEVER CI (UNLC)</t>
+          <t>ORAGROUP TOGO (ORGT)</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>-2.44</v>
+        <v>-2.88</v>
       </c>
       <c r="E31" t="n">
-        <v>3.72</v>
+        <v>-2.88</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1332,27 +1332,27 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NEI-CEDA CI (NEIC)</t>
+          <t>BICI CI (BICC)</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>-2.63</v>
+        <v>-4.12</v>
       </c>
       <c r="E32" t="n">
-        <v>-2.65</v>
+        <v>-4.12</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1361,27 +1361,27 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>👀 À surveiller</t>
+          <t>➖ Neutre</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ORAGROUP TOGO (ORGT)</t>
+          <t>SUCRIVOIRE (SCRC)</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>-2.88</v>
+        <v>-4.79</v>
       </c>
       <c r="E33" t="n">
-        <v>-2.88</v>
+        <v>-1.79</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BICI CI (BICC)</t>
+          <t>SOGB CI (SOGC)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1407,10 +1407,10 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>-4.12</v>
+        <v>-5.41</v>
       </c>
       <c r="E34" t="n">
-        <v>-4.12</v>
+        <v>-5.41</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1426,20 +1426,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SUCRIVOIRE (SCRC)</t>
+          <t>NESTLE CI (NTLC)</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>-4.79</v>
+        <v>-6.11</v>
       </c>
       <c r="E35" t="n">
-        <v>-1.79</v>
+        <v>-6.11</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1455,116 +1455,58 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TOTALENERGIES MARKETING CI (TTLC)</t>
+          <t>SAFCA CI (SAFC)</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>-5.04</v>
+        <v>-10.37</v>
       </c>
       <c r="E36" t="n">
-        <v>-5.04</v>
+        <v>-1.64</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>🟡 Observer</t>
+          <t>🔴 Vente</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>➖ Neutre</t>
+          <t>⚠️ Risque de décrochage</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SAFCA CI (SAFC)</t>
+          <t>SAPH CI (SPHC)</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>-10.37</v>
+        <v>-11.87</v>
       </c>
       <c r="E37" t="n">
-        <v>-1.64</v>
+        <v>3.04</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>🔴 Vente</t>
+          <t>🟡 Observer</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>⚠️ Risque de décrochage</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>SOGB CI (SOGC)</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" t="n">
-        <v>-12.91</v>
-      </c>
-      <c r="E38" t="n">
-        <v>-5.41</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>🟡 Observer</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>➖ Neutre</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>SAPH CI (SPHC)</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>3</v>
-      </c>
-      <c r="D39" t="n">
-        <v>-19.36</v>
-      </c>
-      <c r="E39" t="n">
-        <v>3.04</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>🔴 Vente</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>⚠️ Risque de décrochage</t>
+          <t>👀 À surveiller</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1543,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>333612.73</v>
+        <v>65573.38</v>
       </c>
     </row>
     <row r="3">
@@ -1611,7 +1553,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103921.59</v>
+        <v>25994.77</v>
       </c>
     </row>
     <row r="4">
@@ -1621,7 +1563,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>79614.85000000001</v>
+        <v>20678.55</v>
       </c>
     </row>
     <row r="5">
@@ -1631,7 +1573,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60080.07</v>
+        <v>16567.61</v>
       </c>
     </row>
     <row r="6">
@@ -1641,7 +1583,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40830.49</v>
+        <v>12107.85</v>
       </c>
     </row>
     <row r="7">
@@ -1651,7 +1593,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34751.84</v>
+        <v>10703.76</v>
       </c>
     </row>
     <row r="8">
@@ -1661,7 +1603,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29854.2</v>
+        <v>9435.6</v>
       </c>
     </row>
     <row r="9">
@@ -1671,7 +1613,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24509.83</v>
+        <v>8076.84</v>
       </c>
     </row>
     <row r="10">
@@ -1681,7 +1623,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16196.44</v>
+        <v>5840.88</v>
       </c>
     </row>
     <row r="11">
@@ -1691,7 +1633,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8304.059999999999</v>
+        <v>3379.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>